<commit_message>
Updated to latest versions
</commit_message>
<xml_diff>
--- a/src/test/resources/Excel Files/TestData.xlsx
+++ b/src/test/resources/Excel Files/TestData.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE79B2F4-A649-4CE7-A152-990F18CC4CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7341B3C2-2DD8-4973-ADC2-497719AF6072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SignUpTest" sheetId="8" r:id="rId1"/>
-    <sheet name="SearchItem" sheetId="5" r:id="rId2"/>
+    <sheet name="SearchItemTest" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -118,11 +118,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,13 +429,13 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>